<commit_message>
[T-7933][FIX] odoo_2_odoo_data_transfer: many2one validation
</commit_message>
<xml_diff>
--- a/odoo_2_odoo_data_transfer/templates/product_template.xlsx
+++ b/odoo_2_odoo_data_transfer/templates/product_template.xlsx
@@ -1,388 +1,413 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="116">
   <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>local_target_model_id/id</t>
-  </si>
-  <si>
-    <t>remote_source_model_name</t>
-  </si>
-  <si>
-    <t>domain</t>
-  </si>
-  <si>
-    <t>is_many2one_template</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/id</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/remote_source_field</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/local_target_field_id/id</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/relational_migration_method</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/remote_identifier_field</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/local_identifier_field_id/id</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/manual_id_mappings</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/skip_relational_errors</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/one2many_template_id/id</t>
-  </si>
-  <si>
-    <t>transfer_line_ids/related_model</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_1_70131cf1</t>
-  </si>
-  <si>
-    <t>Productos</t>
-  </si>
-  <si>
-    <t>product_tag_pricelist.model_product_template</t>
-  </si>
-  <si>
-    <t>product.template</t>
-  </si>
-  <si>
-    <t>[]</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_1_6686827c</t>
-  </si>
-  <si>
-    <t>sale_ok</t>
-  </si>
-  <si>
-    <t>product.field_product_template__sale_ok</t>
-  </si>
-  <si>
-    <t>Emparejar claves</t>
-  </si>
-  <si>
-    <t>{}</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_2_a9afc9e2</t>
-  </si>
-  <si>
-    <t>purchase_ok</t>
-  </si>
-  <si>
-    <t>product.field_product_template__purchase_ok</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_3_6ceaa5c4</t>
-  </si>
-  <si>
-    <t>product.field_product_template__name</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_4_f82a0da9</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>point_of_sale.field_product_template__detailed_type</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_5_70a10132</t>
-  </si>
-  <si>
-    <t>invoice_policy</t>
-  </si>
-  <si>
-    <t>sale.field_product_template__invoice_policy</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_6_3de979df</t>
-  </si>
-  <si>
-    <t>default_code</t>
-  </si>
-  <si>
-    <t>product.field_product_template__default_code</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_7_541eeba4</t>
-  </si>
-  <si>
-    <t>barcode</t>
-  </si>
-  <si>
-    <t>product.field_product_template__barcode</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_8_cdeaf893</t>
-  </si>
-  <si>
-    <t>list_price</t>
-  </si>
-  <si>
-    <t>product.field_product_template__list_price</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_9_635a10fb</t>
-  </si>
-  <si>
-    <t>taxes_id</t>
-  </si>
-  <si>
-    <t>account.field_product_template__taxes_id</t>
-  </si>
-  <si>
-    <t>account.field_account_tax__description</t>
-  </si>
-  <si>
-    <t>account.tax</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_10_784fbcd5</t>
-  </si>
-  <si>
-    <t>categ_id</t>
-  </si>
-  <si>
-    <t>product.field_product_template__categ_id</t>
-  </si>
-  <si>
-    <t>complete_name</t>
-  </si>
-  <si>
-    <t>product.field_product_category__complete_name</t>
-  </si>
-  <si>
-    <t>{104:369, 218: 764, 221:765}</t>
-  </si>
-  <si>
-    <t>product.category</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_11_11d7b46b</t>
-  </si>
-  <si>
-    <t>tag_ids</t>
-  </si>
-  <si>
-    <t>product.field_product_template__product_tag_ids</t>
-  </si>
-  <si>
-    <t>product.field_product_tag__name</t>
-  </si>
-  <si>
-    <t>product.tag</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_12_1b6e49a1</t>
-  </si>
-  <si>
-    <t>standard_price</t>
-  </si>
-  <si>
-    <t>product.field_product_template__standard_price</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_15_0f2a9db9</t>
-  </si>
-  <si>
-    <t>uom_id</t>
-  </si>
-  <si>
-    <t>product.field_product_template__uom_id</t>
-  </si>
-  <si>
-    <t>uom.field_uom_uom__name</t>
-  </si>
-  <si>
-    <t>uom.uom</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_16_36851fe3</t>
-  </si>
-  <si>
-    <t>uom_po_id</t>
-  </si>
-  <si>
-    <t>product.field_product_template__uom_po_id</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_17_64fb9711</t>
-  </si>
-  <si>
-    <t>product.field_product_template__description</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_19_85326c9a</t>
-  </si>
-  <si>
-    <t>sale_line_warn_msg</t>
-  </si>
-  <si>
-    <t>sale.field_product_template__sale_line_warn_msg</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_23_67a6658c</t>
-  </si>
-  <si>
-    <t>weight</t>
-  </si>
-  <si>
-    <t>product.field_product_template__weight</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_24_0a4846a3</t>
-  </si>
-  <si>
-    <t>volume</t>
-  </si>
-  <si>
-    <t>product.field_product_template__volume</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_25_ca7f4bcc</t>
-  </si>
-  <si>
-    <t>sale_delay</t>
-  </si>
-  <si>
-    <t>stock.field_product_template__sale_delay</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_26_467be9b7</t>
-  </si>
-  <si>
-    <t>purchase_method</t>
-  </si>
-  <si>
-    <t>purchase.field_product_template__purchase_method</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_72_82ede428</t>
-  </si>
-  <si>
-    <t>route_ids</t>
-  </si>
-  <si>
-    <t>purchase_stock.field_product_template__route_ids</t>
-  </si>
-  <si>
-    <t>stock.field_stock_route__name</t>
-  </si>
-  <si>
-    <t>stock.route</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_73_fc24f450</t>
-  </si>
-  <si>
-    <t>tracking</t>
-  </si>
-  <si>
-    <t>stock.field_product_template__tracking</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_117_8dc138e0</t>
-  </si>
-  <si>
-    <t>image_1920</t>
-  </si>
-  <si>
-    <t>product.field_product_template__image_1920</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_122_2876cff6</t>
-  </si>
-  <si>
-    <t>property_stock_inventory</t>
-  </si>
-  <si>
-    <t>stock.field_product_template__property_stock_inventory</t>
-  </si>
-  <si>
-    <t>stock.field_stock_location__complete_name</t>
-  </si>
-  <si>
-    <t>stock.location</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_123_108b05ad</t>
-  </si>
-  <si>
-    <t>property_stock_production</t>
-  </si>
-  <si>
-    <t>stock.field_product_template__property_stock_production</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_168_26b7c6b9</t>
-  </si>
-  <si>
-    <t>product_old_migration_fields.field_product_template__old_product_template_id</t>
-  </si>
-  <si>
-    <t>__export__.odoo_data_transfer_template_line_172_82565ac6</t>
-  </si>
-  <si>
-    <t>active</t>
-  </si>
-  <si>
-    <t>product.field_product_template__active</t>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">local_target_model_id/id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remote_source_model_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">domain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_many2one_template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/remote_source_field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/local_target_field_id/id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/relational_migration_method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/remote_identifier_field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/local_identifier_field_id/id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/manual_id_mappings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/skip_relational_errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/one2many_template_id/id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfer_line_ids/related_model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_1_70131cf1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Productos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product_tag_pricelist.model_product_template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_1_6686827c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sale_ok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__sale_ok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emparejar claves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_2_a9afc9e2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">purchase_ok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__purchase_ok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_3_6ceaa5c4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_4_f82a0da9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__detailed_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_5_70a10132</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invoice_policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sale.field_product_template__invoice_policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_6_3de979df</t>
+  </si>
+  <si>
+    <t xml:space="preserve">default_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__default_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_7_541eeba4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barcode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__barcode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_8_cdeaf893</t>
+  </si>
+  <si>
+    <t xml:space="preserve">list_price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__list_price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_9_635a10fb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">taxes_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account.field_product_template__taxes_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account.field_account_tax__description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account.tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_10_784fbcd5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categ_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__categ_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">complete_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_category__complete_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{104:369, 218: 764, 221:765}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_11_11d7b46b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tag_ids</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__product_tag_ids</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_tag__name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_12_1b6e49a1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">standard_price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__standard_price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_15_0f2a9db9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uom_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__uom_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uom.field_uom_uom__name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uom.uom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_16_36851fe3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uom_po_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__uom_po_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_17_64fb9711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_19_85326c9a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sale_line_warn_msg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sale.field_product_template__sale_line_warn_msg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_23_67a6658c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_24_0a4846a3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_25_ca7f4bcc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sale_delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.field_product_template__sale_delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_26_467be9b7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">purchase_method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">purchase.field_product_template__purchase_method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_72_82ede428</t>
+  </si>
+  <si>
+    <t xml:space="preserve">route_ids</t>
+  </si>
+  <si>
+    <t xml:space="preserve">purchase_stock.field_product_template__route_ids</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.field_stock_route__name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_73_fc24f450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.field_product_template__tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_117_8dc138e0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image_1920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__image_1920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_122_2876cff6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property_stock_inventory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.field_product_template__property_stock_inventory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.field_stock_location__complete_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_123_108b05ad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property_stock_production</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock.field_product_template__property_stock_production</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_168_26b7c6b9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product_old_migration_fields.field_product_template__old_product_template_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__export__.odoo_data_transfer_template_line_172_82565ac6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">active</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product.field_product_template__active</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="General"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -394,7 +419,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -402,316 +427,72 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:Q28"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="17" width="30.7109375" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="1" style="0" width="30.71"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -764,7 +545,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
@@ -783,7 +564,8 @@
       <c r="F2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="2" t="b">
+      <c r="G2" s="3" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -804,12 +586,13 @@
         <v>26</v>
       </c>
       <c r="O2" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -835,12 +618,13 @@
         <v>26</v>
       </c>
       <c r="O3" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -866,12 +650,13 @@
         <v>26</v>
       </c>
       <c r="O4" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -897,12 +682,13 @@
         <v>26</v>
       </c>
       <c r="O5" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -928,12 +714,13 @@
         <v>26</v>
       </c>
       <c r="O6" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -959,12 +746,13 @@
         <v>26</v>
       </c>
       <c r="O7" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -990,12 +778,13 @@
         <v>26</v>
       </c>
       <c r="O8" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1021,12 +810,13 @@
         <v>26</v>
       </c>
       <c r="O9" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1056,6 +846,7 @@
         <v>26</v>
       </c>
       <c r="O10" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P10" s="2"/>
@@ -1063,7 +854,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1093,6 +884,7 @@
         <v>57</v>
       </c>
       <c r="O11" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P11" s="2"/>
@@ -1100,7 +892,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1130,6 +922,7 @@
         <v>26</v>
       </c>
       <c r="O12" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P12" s="2"/>
@@ -1137,7 +930,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1163,12 +956,13 @@
         <v>26</v>
       </c>
       <c r="O13" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1198,6 +992,7 @@
         <v>26</v>
       </c>
       <c r="O14" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P14" s="2"/>
@@ -1205,7 +1000,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1235,6 +1030,7 @@
         <v>26</v>
       </c>
       <c r="O15" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P15" s="2"/>
@@ -1242,7 +1038,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1268,12 +1064,13 @@
         <v>26</v>
       </c>
       <c r="O16" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1299,12 +1096,13 @@
         <v>26</v>
       </c>
       <c r="O17" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1330,12 +1128,13 @@
         <v>26</v>
       </c>
       <c r="O18" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1361,12 +1160,13 @@
         <v>26</v>
       </c>
       <c r="O19" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1392,12 +1192,13 @@
         <v>26</v>
       </c>
       <c r="O20" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1423,12 +1224,13 @@
         <v>26</v>
       </c>
       <c r="O21" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1458,6 +1260,7 @@
         <v>26</v>
       </c>
       <c r="O22" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P22" s="2"/>
@@ -1465,7 +1268,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1491,12 +1294,13 @@
         <v>26</v>
       </c>
       <c r="O23" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P23" s="2"/>
       <c r="Q23" s="2"/>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1522,12 +1326,13 @@
         <v>26</v>
       </c>
       <c r="O24" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1557,6 +1362,7 @@
         <v>26</v>
       </c>
       <c r="O25" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P25" s="2"/>
@@ -1564,7 +1370,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:17">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1594,6 +1400,7 @@
         <v>26</v>
       </c>
       <c r="O26" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P26" s="2"/>
@@ -1601,7 +1408,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:17">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1627,12 +1434,13 @@
         <v>26</v>
       </c>
       <c r="O27" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
     </row>
-    <row r="28" spans="1:17">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1658,12 +1466,19 @@
         <v>26</v>
       </c>
       <c r="O28" s="2" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="P28" s="2"/>
       <c r="Q28" s="2"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>